<commit_message>
auto: 更新 US Swing 2026-08-01
</commit_message>
<xml_diff>
--- a/hk_swing_pattern/US_Swing_Pattern.xlsx
+++ b/hk_swing_pattern/US_Swing_Pattern.xlsx
@@ -660,9 +660,7 @@
       <c r="N2" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="O2" s="2" t="n">
-        <v>1</v>
-      </c>
+      <c r="O2" s="2" t="inlineStr"/>
       <c r="P2" s="2" t="inlineStr"/>
       <c r="Q2" s="2" t="inlineStr"/>
       <c r="R2" s="2" t="inlineStr">
@@ -1466,7 +1464,7 @@
         <v>14.68</v>
       </c>
       <c r="D16" s="2" t="n">
-        <v>89.7</v>
+        <v>86.73999999999999</v>
       </c>
       <c r="E16" s="2" t="inlineStr"/>
       <c r="F16" s="2" t="inlineStr"/>
@@ -1480,29 +1478,35 @@
       <c r="N16" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="O16" s="2" t="inlineStr"/>
+      <c r="O16" s="2" t="n">
+        <v>1</v>
+      </c>
       <c r="P16" s="2" t="inlineStr"/>
       <c r="Q16" s="2" t="inlineStr"/>
-      <c r="R16" s="2" t="n">
-        <v>-1</v>
+      <c r="R16" s="2" t="inlineStr">
+        <is>
+          <t>预1</t>
+        </is>
       </c>
       <c r="S16" s="2" t="inlineStr"/>
-      <c r="T16" s="2" t="inlineStr"/>
+      <c r="T16" s="2" t="n">
+        <v>0</v>
+      </c>
       <c r="U16" s="2" t="inlineStr"/>
       <c r="V16" s="2" t="n">
-        <v>9.609999999999999</v>
+        <v>8.31</v>
       </c>
       <c r="W16" s="2" t="n">
-        <v>-2.75</v>
+        <v>-2.74</v>
       </c>
       <c r="X16" s="2" t="n">
-        <v>4.78</v>
+        <v>4.8</v>
       </c>
       <c r="Y16" s="2" t="n">
-        <v>-0.9399999999999999</v>
+        <v>-0.92</v>
       </c>
       <c r="Z16" s="2" t="n">
-        <v>1.47</v>
+        <v>1.49</v>
       </c>
     </row>
     <row r="17">
@@ -2758,19 +2762,19 @@
       <c r="T38" s="2" t="inlineStr"/>
       <c r="U38" s="2" t="inlineStr"/>
       <c r="V38" s="2" t="n">
-        <v>-12.6</v>
+        <v>-13.2</v>
       </c>
       <c r="W38" s="2" t="n">
-        <v>-16.96</v>
+        <v>-16.95</v>
       </c>
       <c r="X38" s="2" t="n">
-        <v>-18.1</v>
+        <v>-18.09</v>
       </c>
       <c r="Y38" s="2" t="n">
-        <v>-0.83</v>
+        <v>-0.82</v>
       </c>
       <c r="Z38" s="2" t="n">
-        <v>-1.32</v>
+        <v>-1.31</v>
       </c>
     </row>
     <row r="39">
@@ -4160,9 +4164,7 @@
       <c r="N63" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="O63" s="2" t="n">
-        <v>1</v>
-      </c>
+      <c r="O63" s="2" t="inlineStr"/>
       <c r="P63" s="2" t="inlineStr"/>
       <c r="Q63" s="2" t="inlineStr"/>
       <c r="R63" s="2" t="inlineStr">
@@ -4424,7 +4426,7 @@
         <v>66.44</v>
       </c>
       <c r="D68" s="2" t="n">
-        <v>2.98</v>
+        <v>3.01</v>
       </c>
       <c r="E68" s="2" t="inlineStr"/>
       <c r="F68" s="2" t="inlineStr">
@@ -4488,7 +4490,7 @@
         <v>65.31</v>
       </c>
       <c r="D69" s="2" t="n">
-        <v>111.13</v>
+        <v>111.11</v>
       </c>
       <c r="E69" s="2" t="inlineStr"/>
       <c r="F69" s="2" t="inlineStr">
@@ -5086,17 +5088,17 @@
       </c>
       <c r="S79" s="2" t="inlineStr"/>
       <c r="T79" s="2" t="n">
-        <v>1</v>
+        <v>-1</v>
       </c>
       <c r="U79" s="2" t="inlineStr"/>
       <c r="V79" s="2" t="n">
-        <v>58.7</v>
+        <v>58.6</v>
       </c>
       <c r="W79" s="2" t="n">
         <v>22.42</v>
       </c>
       <c r="X79" s="2" t="n">
-        <v>26.38</v>
+        <v>26.39</v>
       </c>
       <c r="Y79" s="2" t="n">
         <v>-0.78</v>
@@ -7096,7 +7098,7 @@
         <v>95.01000000000001</v>
       </c>
       <c r="D114" s="2" t="n">
-        <v>-2.66</v>
+        <v>-2.67</v>
       </c>
       <c r="E114" s="2" t="inlineStr"/>
       <c r="F114" s="2" t="inlineStr"/>
@@ -7514,7 +7516,7 @@
         <v>-13</v>
       </c>
       <c r="N121" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O121" s="2" t="inlineStr"/>
       <c r="P121" s="2" t="inlineStr"/>
@@ -8046,7 +8048,7 @@
       <c r="L130" s="2" t="inlineStr"/>
       <c r="M130" s="2" t="inlineStr"/>
       <c r="N130" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O130" s="2" t="inlineStr"/>
       <c r="P130" s="2" t="inlineStr"/>
@@ -9406,7 +9408,7 @@
         <v>-9</v>
       </c>
       <c r="N153" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O153" s="2" t="inlineStr"/>
       <c r="P153" s="2" t="inlineStr"/>
@@ -11982,7 +11984,7 @@
         <v>9</v>
       </c>
       <c r="N198" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O198" s="2" t="inlineStr"/>
       <c r="P198" s="2" t="inlineStr"/>
@@ -12500,7 +12502,7 @@
       <c r="L207" s="2" t="inlineStr"/>
       <c r="M207" s="2" t="inlineStr"/>
       <c r="N207" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O207" s="2" t="inlineStr"/>
       <c r="P207" s="2" t="inlineStr"/>
@@ -14928,7 +14930,9 @@
       </c>
       <c r="O248" s="2" t="inlineStr"/>
       <c r="P248" s="2" t="inlineStr"/>
-      <c r="Q248" s="2" t="inlineStr"/>
+      <c r="Q248" s="2" t="n">
+        <v>1</v>
+      </c>
       <c r="R248" s="2" t="n">
         <v>-1</v>
       </c>
@@ -16927,26 +16931,28 @@
       <c r="O282" s="2" t="inlineStr"/>
       <c r="P282" s="2" t="inlineStr"/>
       <c r="Q282" s="2" t="inlineStr"/>
-      <c r="R282" s="2" t="n">
-        <v>-1</v>
+      <c r="R282" s="2" t="inlineStr">
+        <is>
+          <t>预1</t>
+        </is>
       </c>
       <c r="S282" s="2" t="inlineStr"/>
       <c r="T282" s="2" t="inlineStr"/>
       <c r="U282" s="2" t="inlineStr"/>
       <c r="V282" s="2" t="n">
-        <v>12.44</v>
+        <v>11.61</v>
       </c>
       <c r="W282" s="2" t="n">
-        <v>-4.43</v>
+        <v>-4.42</v>
       </c>
       <c r="X282" s="2" t="n">
-        <v>3</v>
+        <v>3.01</v>
       </c>
       <c r="Y282" s="2" t="n">
-        <v>-5.93</v>
+        <v>-5.92</v>
       </c>
       <c r="Z282" s="2" t="n">
-        <v>-9.44</v>
+        <v>-9.42</v>
       </c>
     </row>
     <row r="283">
@@ -18124,9 +18130,7 @@
       <c r="N303" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="O303" s="2" t="n">
-        <v>1</v>
-      </c>
+      <c r="O303" s="2" t="inlineStr"/>
       <c r="P303" s="2" t="inlineStr"/>
       <c r="Q303" s="2" t="inlineStr"/>
       <c r="R303" s="2" t="inlineStr">
@@ -18238,7 +18242,7 @@
         <v>-9</v>
       </c>
       <c r="N305" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O305" s="2" t="inlineStr"/>
       <c r="P305" s="2" t="inlineStr"/>
@@ -18573,10 +18577,10 @@
         </is>
       </c>
       <c r="C311" s="2" t="n">
-        <v>22.67</v>
+        <v>23.25</v>
       </c>
       <c r="D311" s="2" t="n">
-        <v>-0.77</v>
+        <v>1.48</v>
       </c>
       <c r="E311" s="2" t="inlineStr"/>
       <c r="F311" s="2" t="inlineStr"/>
@@ -18600,19 +18604,19 @@
       <c r="T311" s="2" t="inlineStr"/>
       <c r="U311" s="2" t="inlineStr"/>
       <c r="V311" s="2" t="n">
-        <v>109.2</v>
+        <v>110.17</v>
       </c>
       <c r="W311" s="2" t="n">
-        <v>48.2</v>
+        <v>51.97</v>
       </c>
       <c r="X311" s="2" t="n">
-        <v>41.85</v>
+        <v>45.46</v>
       </c>
       <c r="Y311" s="2" t="n">
-        <v>-19.7</v>
+        <v>-15.93</v>
       </c>
       <c r="Z311" s="2" t="n">
-        <v>-87.27</v>
+        <v>-83.5</v>
       </c>
     </row>
     <row r="312">
@@ -18894,19 +18898,19 @@
       <c r="T316" s="2" t="inlineStr"/>
       <c r="U316" s="2" t="inlineStr"/>
       <c r="V316" s="2" t="n">
-        <v>41.97</v>
+        <v>41.31</v>
       </c>
       <c r="W316" s="2" t="n">
-        <v>10.76</v>
+        <v>10.77</v>
       </c>
       <c r="X316" s="2" t="n">
-        <v>10.76</v>
+        <v>10.77</v>
       </c>
       <c r="Y316" s="2" t="n">
-        <v>-3.31</v>
+        <v>-3.29</v>
       </c>
       <c r="Z316" s="2" t="n">
-        <v>-3.99</v>
+        <v>-3.98</v>
       </c>
     </row>
     <row r="317">
@@ -19670,7 +19674,7 @@
         <v>44.43</v>
       </c>
       <c r="D330" s="2" t="n">
-        <v>2.7</v>
+        <v>7.31</v>
       </c>
       <c r="E330" s="2" t="inlineStr"/>
       <c r="F330" s="2" t="inlineStr"/>
@@ -19696,19 +19700,19 @@
       </c>
       <c r="U330" s="2" t="inlineStr"/>
       <c r="V330" s="2" t="n">
-        <v>9.029999999999999</v>
+        <v>8.32</v>
       </c>
       <c r="W330" s="2" t="n">
-        <v>-6.97</v>
+        <v>-6.96</v>
       </c>
       <c r="X330" s="2" t="n">
-        <v>0.29</v>
+        <v>0.3</v>
       </c>
       <c r="Y330" s="2" t="n">
-        <v>-5.02</v>
+        <v>-5.01</v>
       </c>
       <c r="Z330" s="2" t="n">
-        <v>-6.52</v>
+        <v>-6.51</v>
       </c>
     </row>
     <row r="331">
@@ -20071,7 +20075,7 @@
         </is>
       </c>
       <c r="C337" s="2" t="n">
-        <v>11.84</v>
+        <v>11.82</v>
       </c>
       <c r="D337" s="2" t="n">
         <v>28.92</v>
@@ -20098,19 +20102,19 @@
         <v>1</v>
       </c>
       <c r="V337" s="2" t="n">
-        <v>-63.02</v>
+        <v>-63.06</v>
       </c>
       <c r="W337" s="2" t="n">
-        <v>-31.04</v>
+        <v>-31.16</v>
       </c>
       <c r="X337" s="2" t="n">
-        <v>-20.37</v>
+        <v>-20.51</v>
       </c>
       <c r="Y337" s="2" t="n">
-        <v>7.2</v>
+        <v>7.09</v>
       </c>
       <c r="Z337" s="2" t="n">
-        <v>7.86</v>
+        <v>7.75</v>
       </c>
     </row>
     <row r="338">
@@ -20517,19 +20521,21 @@
       <c r="S344" s="2" t="n">
         <v>-1</v>
       </c>
-      <c r="T344" s="2" t="inlineStr"/>
+      <c r="T344" s="2" t="n">
+        <v>-1</v>
+      </c>
       <c r="U344" s="2" t="inlineStr"/>
       <c r="V344" s="2" t="n">
-        <v>18.94</v>
+        <v>18.46</v>
       </c>
       <c r="W344" s="2" t="n">
-        <v>-0.89</v>
+        <v>-0.88</v>
       </c>
       <c r="X344" s="2" t="n">
-        <v>0.02</v>
+        <v>0.03</v>
       </c>
       <c r="Y344" s="2" t="n">
-        <v>-3.41</v>
+        <v>-3.4</v>
       </c>
       <c r="Z344" s="2" t="n">
         <v>0.24</v>
@@ -22772,7 +22778,7 @@
       <c r="L383" s="2" t="inlineStr"/>
       <c r="M383" s="2" t="inlineStr"/>
       <c r="N383" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O383" s="2" t="inlineStr"/>
       <c r="P383" s="2" t="inlineStr"/>
@@ -23836,9 +23842,7 @@
       <c r="N401" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="O401" s="2" t="n">
-        <v>1</v>
-      </c>
+      <c r="O401" s="2" t="inlineStr"/>
       <c r="P401" s="2" t="inlineStr"/>
       <c r="Q401" s="2" t="inlineStr"/>
       <c r="R401" s="2" t="n">
@@ -25192,7 +25196,7 @@
         <v>-9</v>
       </c>
       <c r="N425" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O425" s="2" t="inlineStr"/>
       <c r="P425" s="2" t="inlineStr"/>
@@ -25528,7 +25532,7 @@
       <c r="L431" s="2" t="inlineStr"/>
       <c r="M431" s="2" t="inlineStr"/>
       <c r="N431" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O431" s="2" t="inlineStr"/>
       <c r="P431" s="2" t="inlineStr"/>
@@ -25900,19 +25904,19 @@
       <c r="T437" s="2" t="inlineStr"/>
       <c r="U437" s="2" t="inlineStr"/>
       <c r="V437" s="2" t="n">
-        <v>65.56999999999999</v>
+        <v>64.98</v>
       </c>
       <c r="W437" s="2" t="n">
-        <v>20.02</v>
+        <v>20.03</v>
       </c>
       <c r="X437" s="2" t="n">
-        <v>10.28</v>
+        <v>10.29</v>
       </c>
       <c r="Y437" s="2" t="n">
-        <v>-6.49</v>
+        <v>-6.48</v>
       </c>
       <c r="Z437" s="2" t="n">
-        <v>2.08</v>
+        <v>2.09</v>
       </c>
     </row>
     <row r="438">
@@ -26526,7 +26530,7 @@
         <v>275.74</v>
       </c>
       <c r="D448" s="2" t="n">
-        <v>-7</v>
+        <v>-5.54</v>
       </c>
       <c r="E448" s="2" t="inlineStr"/>
       <c r="F448" s="2" t="inlineStr"/>
@@ -26550,19 +26554,19 @@
       <c r="T448" s="2" t="inlineStr"/>
       <c r="U448" s="2" t="inlineStr"/>
       <c r="V448" s="2" t="n">
-        <v>61.03</v>
+        <v>60.36</v>
       </c>
       <c r="W448" s="2" t="n">
-        <v>18.44</v>
+        <v>18.46</v>
       </c>
       <c r="X448" s="2" t="n">
-        <v>11.11</v>
+        <v>11.12</v>
       </c>
       <c r="Y448" s="2" t="n">
-        <v>-3</v>
+        <v>-2.99</v>
       </c>
       <c r="Z448" s="2" t="n">
-        <v>-9.26</v>
+        <v>-9.24</v>
       </c>
     </row>
     <row r="449">
@@ -27058,7 +27062,7 @@
       <c r="L457" s="2" t="inlineStr"/>
       <c r="M457" s="2" t="inlineStr"/>
       <c r="N457" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O457" s="2" t="inlineStr"/>
       <c r="P457" s="2" t="inlineStr"/>
@@ -27366,19 +27370,19 @@
       <c r="T462" s="2" t="inlineStr"/>
       <c r="U462" s="2" t="inlineStr"/>
       <c r="V462" s="2" t="n">
-        <v>90.34999999999999</v>
+        <v>89.77</v>
       </c>
       <c r="W462" s="2" t="n">
-        <v>42.84</v>
+        <v>42.85</v>
       </c>
       <c r="X462" s="2" t="n">
-        <v>31.28</v>
+        <v>31.29</v>
       </c>
       <c r="Y462" s="2" t="n">
-        <v>1.92</v>
+        <v>1.93</v>
       </c>
       <c r="Z462" s="2" t="n">
-        <v>14.81</v>
+        <v>14.82</v>
       </c>
     </row>
     <row r="463">
@@ -27456,7 +27460,7 @@
         <v>268.57</v>
       </c>
       <c r="D464" s="2" t="n">
-        <v>2.8</v>
+        <v>3.13</v>
       </c>
       <c r="E464" s="2" t="inlineStr"/>
       <c r="F464" s="2" t="inlineStr"/>
@@ -29074,7 +29078,7 @@
         <v>293.82</v>
       </c>
       <c r="D492" s="2" t="n">
-        <v>99.31999999999999</v>
+        <v>99.31</v>
       </c>
       <c r="E492" s="2" t="inlineStr">
         <is>
@@ -30022,7 +30026,7 @@
         <v>762.63</v>
       </c>
       <c r="D510" s="2" t="n">
-        <v>108.4</v>
+        <v>108.36</v>
       </c>
       <c r="E510" s="2" t="inlineStr"/>
       <c r="F510" s="2" t="inlineStr"/>

</xml_diff>

<commit_message>
auto: 更新 US Swing 2026-08-09
</commit_message>
<xml_diff>
--- a/hk_swing_pattern/US_Swing_Pattern.xlsx
+++ b/hk_swing_pattern/US_Swing_Pattern.xlsx
@@ -8278,14 +8278,20 @@
         <v>209.7</v>
       </c>
       <c r="D134" s="2" t="n">
-        <v>107.48</v>
+        <v>108.06</v>
       </c>
       <c r="E134" s="2" t="inlineStr"/>
-      <c r="F134" s="2" t="inlineStr"/>
+      <c r="F134" s="2" t="inlineStr">
+        <is>
+          <t>顶背离</t>
+        </is>
+      </c>
       <c r="G134" s="2" t="inlineStr"/>
       <c r="H134" s="2" t="inlineStr"/>
       <c r="I134" s="2" t="inlineStr"/>
-      <c r="J134" s="2" t="inlineStr"/>
+      <c r="J134" s="2" t="n">
+        <v>-1</v>
+      </c>
       <c r="K134" s="2" t="inlineStr"/>
       <c r="L134" s="2" t="n">
         <v>-9</v>
@@ -8297,27 +8303,27 @@
       <c r="O134" s="2" t="inlineStr"/>
       <c r="P134" s="2" t="inlineStr"/>
       <c r="Q134" s="2" t="inlineStr"/>
-      <c r="R134" s="2" t="inlineStr">
-        <is>
-          <t>预1</t>
-        </is>
-      </c>
-      <c r="S134" s="2" t="inlineStr"/>
+      <c r="R134" s="2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="S134" s="2" t="n">
+        <v>-1</v>
+      </c>
       <c r="T134" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="U134" s="2" t="inlineStr"/>
       <c r="V134" s="2" t="n">
-        <v>6.08</v>
+        <v>6.42</v>
       </c>
       <c r="W134" s="2" t="n">
         <v>-5.26</v>
       </c>
       <c r="X134" s="2" t="n">
-        <v>8.56</v>
+        <v>8.550000000000001</v>
       </c>
       <c r="Y134" s="2" t="n">
-        <v>-5.06</v>
+        <v>-5.07</v>
       </c>
       <c r="Z134" s="2" t="n">
         <v>-1.78</v>
@@ -30523,7 +30529,7 @@
     <row r="2">
       <c r="A2" s="4" t="inlineStr">
         <is>
-          <t>截至: 2026-08-08 | 523 只</t>
+          <t>截至: 2026-08-09 | 523 只</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: 更新 US Swing 2026-08-16
</commit_message>
<xml_diff>
--- a/hk_swing_pattern/US_Swing_Pattern.xlsx
+++ b/hk_swing_pattern/US_Swing_Pattern.xlsx
@@ -1412,7 +1412,7 @@
         <v>-3.43</v>
       </c>
       <c r="X15" s="2" t="n">
-        <v>-1.77</v>
+        <v>-1.76</v>
       </c>
       <c r="Y15" s="2" t="n">
         <v>-2.85</v>
@@ -5592,7 +5592,7 @@
         <v>101.3</v>
       </c>
       <c r="D88" s="2" t="n">
-        <v>80.3</v>
+        <v>84.89</v>
       </c>
       <c r="E88" s="2" t="inlineStr"/>
       <c r="F88" s="2" t="inlineStr"/>
@@ -5602,7 +5602,9 @@
       <c r="J88" s="2" t="inlineStr"/>
       <c r="K88" s="2" t="inlineStr"/>
       <c r="L88" s="2" t="inlineStr"/>
-      <c r="M88" s="2" t="inlineStr"/>
+      <c r="M88" s="2" t="n">
+        <v>-9</v>
+      </c>
       <c r="N88" s="2" t="n">
         <v>1</v>
       </c>
@@ -5621,10 +5623,10 @@
         <v>22.39</v>
       </c>
       <c r="W88" s="2" t="n">
-        <v>-2.34</v>
+        <v>-2.33</v>
       </c>
       <c r="X88" s="2" t="n">
-        <v>3.28</v>
+        <v>3.29</v>
       </c>
       <c r="Y88" s="2" t="n">
         <v>-1.78</v>
@@ -9748,9 +9750,7 @@
       <c r="J159" s="2" t="inlineStr"/>
       <c r="K159" s="2" t="inlineStr"/>
       <c r="L159" s="2" t="inlineStr"/>
-      <c r="M159" s="2" t="n">
-        <v>-9</v>
-      </c>
+      <c r="M159" s="2" t="inlineStr"/>
       <c r="N159" s="2" t="n">
         <v>1</v>
       </c>
@@ -9769,16 +9769,16 @@
         <v>29.84</v>
       </c>
       <c r="W159" s="2" t="n">
-        <v>5.46</v>
+        <v>5.44</v>
       </c>
       <c r="X159" s="2" t="n">
-        <v>4.32</v>
+        <v>4.31</v>
       </c>
       <c r="Y159" s="2" t="n">
         <v>3.08</v>
       </c>
       <c r="Z159" s="2" t="n">
-        <v>12.35</v>
+        <v>12.33</v>
       </c>
     </row>
     <row r="160">
@@ -13454,19 +13454,19 @@
       <c r="T223" s="2" t="inlineStr"/>
       <c r="U223" s="2" t="inlineStr"/>
       <c r="V223" s="2" t="n">
-        <v>47.1</v>
+        <v>47.09</v>
       </c>
       <c r="W223" s="2" t="n">
-        <v>12.96</v>
+        <v>12.95</v>
       </c>
       <c r="X223" s="2" t="n">
-        <v>11.99</v>
+        <v>11.98</v>
       </c>
       <c r="Y223" s="2" t="n">
         <v>1.86</v>
       </c>
       <c r="Z223" s="2" t="n">
-        <v>-0.33</v>
+        <v>-0.35</v>
       </c>
     </row>
     <row r="224">
@@ -14162,7 +14162,7 @@
         <v>83.34</v>
       </c>
       <c r="D236" s="2" t="n">
-        <v>106.75</v>
+        <v>106.76</v>
       </c>
       <c r="E236" s="2" t="inlineStr"/>
       <c r="F236" s="2" t="inlineStr"/>
@@ -14662,19 +14662,19 @@
         <v>1</v>
       </c>
       <c r="V244" s="2" t="n">
-        <v>70.62</v>
+        <v>70.58</v>
       </c>
       <c r="W244" s="2" t="n">
-        <v>21.01</v>
+        <v>20.96</v>
       </c>
       <c r="X244" s="2" t="n">
-        <v>9.41</v>
+        <v>9.359999999999999</v>
       </c>
       <c r="Y244" s="2" t="n">
-        <v>6.22</v>
+        <v>6.21</v>
       </c>
       <c r="Z244" s="2" t="n">
-        <v>14.58</v>
+        <v>14.53</v>
       </c>
     </row>
     <row r="245">
@@ -19304,19 +19304,19 @@
       <c r="T324" s="2" t="inlineStr"/>
       <c r="U324" s="2" t="inlineStr"/>
       <c r="V324" s="2" t="n">
-        <v>89.52</v>
+        <v>89.51000000000001</v>
       </c>
       <c r="W324" s="2" t="n">
-        <v>30.6</v>
+        <v>30.59</v>
       </c>
       <c r="X324" s="2" t="n">
-        <v>33.98</v>
+        <v>33.97</v>
       </c>
       <c r="Y324" s="2" t="n">
         <v>-3.66</v>
       </c>
       <c r="Z324" s="2" t="n">
-        <v>6.11</v>
+        <v>6.1</v>
       </c>
     </row>
     <row r="325">
@@ -22932,7 +22932,7 @@
         <v>3.31</v>
       </c>
       <c r="Z385" s="2" t="n">
-        <v>5.7</v>
+        <v>5.69</v>
       </c>
     </row>
     <row r="386">
@@ -24823,16 +24823,16 @@
         <v>27.15</v>
       </c>
       <c r="W418" s="2" t="n">
-        <v>0.4</v>
+        <v>0.41</v>
       </c>
       <c r="X418" s="2" t="n">
-        <v>2.14</v>
+        <v>2.15</v>
       </c>
       <c r="Y418" s="2" t="n">
         <v>1.96</v>
       </c>
       <c r="Z418" s="2" t="n">
-        <v>-2.42</v>
+        <v>-2.41</v>
       </c>
     </row>
     <row r="419">
@@ -25204,7 +25204,7 @@
         <v>358.52</v>
       </c>
       <c r="D425" s="2" t="n">
-        <v>14.58</v>
+        <v>85.81</v>
       </c>
       <c r="E425" s="2" t="inlineStr"/>
       <c r="F425" s="2" t="inlineStr"/>
@@ -25228,19 +25228,19 @@
       <c r="T425" s="2" t="inlineStr"/>
       <c r="U425" s="2" t="inlineStr"/>
       <c r="V425" s="2" t="n">
-        <v>14.87</v>
+        <v>14.86</v>
       </c>
       <c r="W425" s="2" t="n">
-        <v>-13.7</v>
+        <v>-13.74</v>
       </c>
       <c r="X425" s="2" t="n">
-        <v>-20.22</v>
+        <v>-20.25</v>
       </c>
       <c r="Y425" s="2" t="n">
         <v>3.97</v>
       </c>
       <c r="Z425" s="2" t="n">
-        <v>-18.37</v>
+        <v>-18.41</v>
       </c>
     </row>
     <row r="426">
@@ -29560,7 +29560,7 @@
         <v>181</v>
       </c>
       <c r="D502" s="2" t="n">
-        <v>72.39</v>
+        <v>71.77</v>
       </c>
       <c r="E502" s="2" t="inlineStr"/>
       <c r="F502" s="2" t="inlineStr"/>
@@ -29582,10 +29582,10 @@
       <c r="T502" s="2" t="inlineStr"/>
       <c r="U502" s="2" t="inlineStr"/>
       <c r="V502" s="2" t="n">
-        <v>40.42</v>
+        <v>40.43</v>
       </c>
       <c r="W502" s="2" t="n">
-        <v>9.300000000000001</v>
+        <v>9.31</v>
       </c>
       <c r="X502" s="2" t="n">
         <v>11.07</v>
@@ -29716,7 +29716,7 @@
         <v>96.7</v>
       </c>
       <c r="D505" s="2" t="n">
-        <v>114.31</v>
+        <v>113.23</v>
       </c>
       <c r="E505" s="2" t="inlineStr"/>
       <c r="F505" s="2" t="inlineStr"/>
@@ -29738,19 +29738,19 @@
       <c r="T505" s="2" t="inlineStr"/>
       <c r="U505" s="2" t="inlineStr"/>
       <c r="V505" s="2" t="n">
-        <v>31.79</v>
+        <v>31.76</v>
       </c>
       <c r="W505" s="2" t="n">
-        <v>1.42</v>
+        <v>1.36</v>
       </c>
       <c r="X505" s="2" t="n">
-        <v>12.38</v>
+        <v>12.3</v>
       </c>
       <c r="Y505" s="2" t="n">
         <v>2.88</v>
       </c>
       <c r="Z505" s="2" t="n">
-        <v>11.95</v>
+        <v>11.89</v>
       </c>
     </row>
     <row r="506">
@@ -29848,7 +29848,7 @@
         <v>-6.4</v>
       </c>
       <c r="X507" s="2" t="n">
-        <v>-7.28</v>
+        <v>-7.29</v>
       </c>
       <c r="Y507" s="2" t="n">
         <v>-4.82</v>
@@ -30682,13 +30682,13 @@
       <c r="T523" s="2" t="inlineStr"/>
       <c r="U523" s="2" t="inlineStr"/>
       <c r="V523" s="2" t="n">
-        <v>28.39</v>
+        <v>28.38</v>
       </c>
       <c r="W523" s="2" t="n">
-        <v>1.15</v>
+        <v>1.14</v>
       </c>
       <c r="X523" s="2" t="n">
-        <v>-7.3</v>
+        <v>-7.31</v>
       </c>
       <c r="Y523" s="2" t="n">
         <v>5.97</v>
@@ -30777,7 +30777,7 @@
     <row r="2">
       <c r="A2" s="4" t="inlineStr">
         <is>
-          <t>截至: 2026-08-15 | 523 只</t>
+          <t>截至: 2026-08-16 | 523 只</t>
         </is>
       </c>
     </row>

</xml_diff>